<commit_message>
docs: insert Zenodo DOI into IJIR submission package
</commit_message>
<xml_diff>
--- a/06_manuscript/ijir_v0_1_20260720/05_tables/IJIR_Table_1_Data_Sources_v0_1.xlsx
+++ b/06_manuscript/ijir_v0_1_20260720/05_tables/IJIR_Table_1_Data_Sources_v0_1.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table" sheetId="1" r:id="Rc657c4f6e6594789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table" sheetId="1" r:id="R4c4e9abfff5042a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -519,7 +519,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R908190e1357c45ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re43265cee0094cbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>